<commit_message>
SA-21 phần 1: điền nhãn chấm bài giảng của C1 (do Claude chấm)
Chấm 169 bản của 48 khái niệm và 8 bản chấm thử. Ghi chú chung nói rõ
nhãn do AI chấm, quy ước đã dùng và các lỗi hệ thống thấy được.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRQ8Jy5gH99KhJEVjVBKvL
</commit_message>
<xml_diff>
--- a/danh-gia-pha-b/sa21-giao-nguoi-cham/phan-1/thu-sa21-C1.xlsx
+++ b/danh-gia-pha-b/sa21-giao-nguoi-cham/phan-1/thu-sa21-C1.xlsx
@@ -633,10 +633,26 @@
       <c r="A14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Giờ Việt Nam (UTC+7). Chấm bằng Claude (AI) theo yêu cầu của chủ dự án, không phải người chấm.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -952,15 +968,31 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="9" t="n"/>
       <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
+      <c r="K2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>diễn giải điều kiện chỉ số bằng lời (dưới/trên đường chéo); thêm ma trận chéo là trường hợp riêng</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -978,15 +1010,39 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D3" s="11" t="n"/>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="11" t="n"/>
-      <c r="G3" s="11" t="n"/>
-      <c r="H3" s="11" t="n"/>
-      <c r="I3" s="11" t="n"/>
+      <c r="D3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>thua</t>
+        </is>
+      </c>
       <c r="J3" s="11" t="n"/>
-      <c r="K3" s="11" t="n"/>
-      <c r="L3" s="11" t="n"/>
+      <c r="K3" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>khối gợi lại chỉ nhắc lại đúng hai định nghĩa mà phần giải thích nói lại; câu nối đưa được ý "gọi chung là ma trận tam giác"</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1004,15 +1060,39 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="11" t="n"/>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="n"/>
-      <c r="I4" s="11" t="n"/>
+      <c r="D4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>thua</t>
+        </is>
+      </c>
       <c r="J4" s="11" t="n"/>
-      <c r="K4" s="11" t="n"/>
-      <c r="L4" s="11" t="n"/>
+      <c r="K4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>giải thích gần như chép lại định nghĩa</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1030,15 +1110,35 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="11" t="n"/>
+      <c r="D5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
       <c r="H5" s="11" t="n"/>
-      <c r="I5" s="11" t="n"/>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>thua</t>
+        </is>
+      </c>
       <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
-      <c r="L5" s="11" t="n"/>
+      <c r="K5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>LOI: hai ý chỉ là mẩu "còn viết" (mất công thức khi trích); phần còn lại chép nguyên văn</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1056,15 +1156,31 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
+      <c r="K6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>khối "Ví dụ" thật ra là thêm một ý giải thích, không phải ví dụ</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1082,15 +1198,39 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="11" t="n"/>
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="J7" s="11" t="n"/>
-      <c r="K7" s="11" t="n"/>
-      <c r="L7" s="11" t="n"/>
+      <c r="K7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>thiếu ý tầng lớp trung gian ngả về phía nào tùy lợi ích</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1108,15 +1248,35 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="D8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
       <c r="H8" s="11" t="n"/>
-      <c r="I8" s="11" t="n"/>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>trung_tinh</t>
+        </is>
+      </c>
       <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
+      <c r="K8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>hai ý đầu nói về giai cấp thống trị và xung đột giai cấp, lạc khỏi khái niệm; bỏ mất ý chính của định nghĩa (không có vị trí cơ bản, thường xuyên bị phân hóa)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1134,15 +1294,39 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="11" t="n"/>
+      <c r="D9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>vua</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>co_ich</t>
+        </is>
+      </c>
       <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="11" t="n"/>
+      <c r="K9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>đủ cả định nghĩa và vai trò của lợi ích; câu nối đặt khái niệm cạnh giai cấp thống trị và bị trị</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1205,19 +1389,31 @@
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="n"/>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>CÔNG KHAI: nhãn trong tệp chấm thử này do Claude (mô hình AI của Anthropic) chấm theo yêu cầu của chủ dự án, không phải người chấm. Luật tóm tắt ghi "không dùng công cụ AI"; đề nghị dùng C1 làm tham chiếu AI hoặc loại khỏi phân tích chính.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="11" t="n"/>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Quy ước dùng giống tệp chấm chính: so_y_sai chỉ đếm ý ngược sách; câu cụt, lạc đề hạ su_pham / doc_duoc và ghi ở ghi_chu; goi_lai_tiep_theo chấm chung hai khối, thua khi khối chỉ nhắc lại điều phần giải thích đã nói.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="n"/>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>T02 D là mục lỗi (LOI): hai ý chỉ còn mẩu "còn viết" vì công thức bị mất khi trích.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">

</xml_diff>